<commit_message>
Add RKEMerkezPage for centralized RKE management interface
- Implemented a new page that combines Inventory, Inspection, and Report tabs.
- Utilized lazy-loaded tabs with QStackedWidget for efficient resource management.
- Enabled data transfer between tabs, specifically from Inventory to Inspection.
- Integrated error handling for module loading failures.
- Added refresh functionality to reload the active tab's data.
</commit_message>
<xml_diff>
--- a/docs/Kitap1.xlsx
+++ b/docs/Kitap1.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Python Program\REPYS-main\REPYS\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Yeni klasör\REPYS\REPYS\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{838FB215-E090-4A29-B96B-6F05DCA3F74C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAF164CE-38CD-4ACA-A320-C4BF7CB3233A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{44CB2DA0-E234-42E2-AC26-CF4EEF4F8844}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{44CB2DA0-E234-42E2-AC26-CF4EEF4F8844}"/>
   </bookViews>
   <sheets>
     <sheet name="Kitap1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sayfa1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Kitap1!$A$1:$AD$187</definedName>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1615" uniqueCount="577">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1633" uniqueCount="580">
   <si>
     <t>KimlikNo</t>
   </si>
@@ -1770,6 +1771,15 @@
   </si>
   <si>
     <t>Acil USG</t>
+  </si>
+  <si>
+    <t>Vatan Yerleşkesi</t>
+  </si>
+  <si>
+    <t>Rapor Sekreteri</t>
+  </si>
+  <si>
+    <t>Acil Ultrasonnografi</t>
   </si>
 </sst>
 </file>
@@ -12223,4 +12233,110 @@
   <autoFilter ref="A1:AD187" xr:uid="{A746B199-E49E-43E0-87C1-78828739847E}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{433154E5-C639-4980-AA55-3709BFB230D6}">
+  <dimension ref="A1:A18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>577</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A22">
+    <sortCondition ref="A2:A22"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>